<commit_message>
feat(160-01): stage delivered codeset (CMP threshold 11, eligible_sex)
- Replace data/reference/surveillance_codeset.xlsx with Phase 160 delivery:
  SC132 min_analyte_count raised 7 -> 11 (full BMP can no longer qualify as CMP)
  Modalities sheet: new eligible_sex column, F on Mammogram and Breast MRI
- Delete root-level surveillance_codeset_160.xlsx (now in place)
- Update data/reference/README.md: document both Phase 160 edits, R/88 invariant (> 8)

Note: Rscript unavailable on Windows host; cell-by-cell diff deferred to HiPerGator
(160-04 Task 2 will run the automated verify command before shipping workbook).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/reference/surveillance_codeset.xlsx
+++ b/data/reference/surveillance_codeset.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -645,6 +645,30 @@
       <c r="B17" s="4" t="inlineStr">
         <is>
           <t>As Phase 158: TSH / Free T4 on Thyroid function rows; "verify" on codes still to confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>eligible_sex (Phase 160)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Modalities column: blank = all-patient figures only; F or M = also report figures among that sex (denominator, percentage, person-year rate) plus counts for other/unknown sex. F on Mammogram and Breast MRI. All-patient figures are never changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Phase 160 change</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-25: CMP analyte_min_same_day min_analyte_count 7 -&gt; 11 (a full BMP, 8 analytes, no longer counts as CMP sensitivity). Modalities gains eligible_sex.</t>
         </is>
       </c>
     </row>
@@ -8566,7 +8590,7 @@
       </c>
       <c r="N133" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -23310,12 +23334,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -23334,6 +23359,11 @@
           <t>display_order</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>eligible_sex</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -23351,6 +23381,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -23368,6 +23403,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -23385,6 +23425,7 @@
           <t>3</t>
         </is>
       </c>
+      <c r="D4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -23402,6 +23443,7 @@
           <t>4</t>
         </is>
       </c>
+      <c r="D5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -23419,6 +23461,7 @@
           <t>5</t>
         </is>
       </c>
+      <c r="D6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -23436,6 +23479,7 @@
           <t>6</t>
         </is>
       </c>
+      <c r="D7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -23453,6 +23497,7 @@
           <t>7</t>
         </is>
       </c>
+      <c r="D8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -23470,6 +23515,7 @@
           <t>8</t>
         </is>
       </c>
+      <c r="D9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -23487,6 +23533,7 @@
           <t>9</t>
         </is>
       </c>
+      <c r="D10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -23504,6 +23551,7 @@
           <t>10</t>
         </is>
       </c>
+      <c r="D11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -23521,6 +23569,7 @@
           <t>11</t>
         </is>
       </c>
+      <c r="D12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -23538,6 +23587,7 @@
           <t>12</t>
         </is>
       </c>
+      <c r="D13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -23555,6 +23605,7 @@
           <t>13</t>
         </is>
       </c>
+      <c r="D14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -23572,6 +23623,7 @@
           <t>14</t>
         </is>
       </c>
+      <c r="D15" s="5" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:C15"/>

</xml_diff>

<commit_message>
feat(160-04): add A3-confirmed CO2/albumin/creatinine codes to Lab_Analytes
LA190 (2026-3, CO2), LA191 (1752-5, ALBUMIN), LA192 (45066-8, CREATININE)
added to surveillance_codeset.xlsx after A3 diagnostic confirmed one source
reports these results under non-standard LOINCs. 1756-6 deliberately not added.
KEY sheet documents the addition. README updated with the codeset-only note.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/reference/surveillance_codeset.xlsx
+++ b/data/reference/surveillance_codeset.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Analysis_Codeset'!$A$1:$N$168</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lab_Analytes'!$A$1:$M$190</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lab_Analytes'!$A$1:$M$193</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lab_Analytes_Excluded'!$A$1:$G$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Modalities'!$A$1:$C$15</definedName>
   </definedNames>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -669,6 +669,18 @@
       <c r="B19" s="4" t="inlineStr">
         <is>
           <t>2026-09-25: CMP analyte_min_same_day min_analyte_count 7 -&gt; 11 (a full BMP, 8 analytes, no longer counts as CMP sensitivity). Modalities gains eligible_sex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Phase 160 additions</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-25: LA190 (2026-3, CO2), LA191 (1752-5, ALBUMIN) and LA192 (45066-8, CREATININE) added after the A3 missing-analyte diagnostic showed one source reporting these results under non-standard LOINCs. Not added: 1756-6 (CSF/serum albumin ratio code, appears alongside 1752-5 on the same days).</t>
         </is>
       </c>
     </row>
@@ -10554,7 +10566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M190"/>
+  <dimension ref="A1:M193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -21670,8 +21682,181 @@
         </is>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>LA190</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>2026-3</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>2026-3</t>
+        </is>
+      </c>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>LAB_RESULT_CM</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="n"/>
+      <c r="H191" s="5" t="inlineStr">
+        <is>
+          <t>Carbon dioxide, total [Moles/volume] in Arterial blood</t>
+        </is>
+      </c>
+      <c r="I191" s="5" t="inlineStr">
+        <is>
+          <t>Carbon dioxide</t>
+        </is>
+      </c>
+      <c r="J191" s="5" t="inlineStr">
+        <is>
+          <t>BldA</t>
+        </is>
+      </c>
+      <c r="K191" s="5" t="n"/>
+      <c r="L191" s="5" t="inlineStr">
+        <is>
+          <t>Arterial-blood LOINC used by one source for serum CO2 (raw name "CO2 CONTENT", mmol/L, same days as anion gap and calculated osmolality); confirmed from A3 2026-09-25</t>
+        </is>
+      </c>
+      <c r="M191" s="5" t="inlineStr">
+        <is>
+          <t>added Phase 160 from A3 missing-analyte diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="5" t="inlineStr">
+        <is>
+          <t>LA191</t>
+        </is>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>ALBUMIN</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="D192" s="5" t="inlineStr">
+        <is>
+          <t>1752-5</t>
+        </is>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>1752-5</t>
+        </is>
+      </c>
+      <c r="F192" s="5" t="inlineStr">
+        <is>
+          <t>LAB_RESULT_CM</t>
+        </is>
+      </c>
+      <c r="G192" s="5" t="n"/>
+      <c r="H192" s="5" t="inlineStr">
+        <is>
+          <t>Albumin [Mass/volume] in Synovial fluid</t>
+        </is>
+      </c>
+      <c r="I192" s="5" t="inlineStr">
+        <is>
+          <t>Albumin</t>
+        </is>
+      </c>
+      <c r="J192" s="5" t="inlineStr">
+        <is>
+          <t>Synv fld</t>
+        </is>
+      </c>
+      <c r="K192" s="5" t="n"/>
+      <c r="L192" s="5" t="inlineStr">
+        <is>
+          <t>Synovial-fluid LOINC used by one source for serum albumin (raw name "ALBUMIN", g/dL, on CMP days); confirmed from A3 2026-09-25</t>
+        </is>
+      </c>
+      <c r="M192" s="5" t="inlineStr">
+        <is>
+          <t>added Phase 160 from A3 missing-analyte diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>LA192</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>CREATININE</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>45066-8</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>45066-8</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>LAB_RESULT_CM</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="n"/>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>Creatinine and Glomerular filtration rate.predicted panel - Serum or Plasma</t>
+        </is>
+      </c>
+      <c r="I193" s="5" t="n"/>
+      <c r="J193" s="5" t="inlineStr">
+        <is>
+          <t>Ser/Plas</t>
+        </is>
+      </c>
+      <c r="K193" s="5" t="n"/>
+      <c r="L193" s="5" t="inlineStr">
+        <is>
+          <t>Panel LOINC carrying the creatinine result (raw name "Creatinine", mg/dL); confirmed from A3 2026-09-25</t>
+        </is>
+      </c>
+      <c r="M193" s="5" t="inlineStr">
+        <is>
+          <t>added Phase 160 from A3 missing-analyte diagnostic</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M190"/>
+  <autoFilter ref="A1:M193"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(160-04): add LA193 (1756-6 albumin) from A3 re-run
LA193 added to Lab_Analytes in surveillance_codeset.xlsx (LOINC 1756-6,
ALBUMIN, LAB_RESULT_CM). A3 re-run showed this code carries serum albumin
(g/dL) on its own days — present on 61% of CMP days still missing albumin
after LA190-LA192. Root copy deleted; README Phase 160 line updated to
cover LA190-LA193 and remove the stale "1756-6 not added" note.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/reference/surveillance_codeset.xlsx
+++ b/data/reference/surveillance_codeset.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Analysis_Codeset'!$A$1:$N$168</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lab_Analytes'!$A$1:$M$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lab_Analytes'!$A$1:$M$194</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lab_Analytes_Excluded'!$A$1:$G$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Modalities'!$A$1:$C$15</definedName>
   </definedNames>
@@ -468,6 +468,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -680,7 +681,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25: LA190 (2026-3, CO2), LA191 (1752-5, ALBUMIN) and LA192 (45066-8, CREATININE) added after the A3 missing-analyte diagnostic showed one source reporting these results under non-standard LOINCs. Not added: 1756-6 (CSF/serum albumin ratio code, appears alongside 1752-5 on the same days).</t>
+          <t>2026-09-25: LA190 (2026-3, CO2), LA191 (1752-5, ALBUMIN) and LA192 (45066-8, CREATININE) added after the A3 missing-analyte diagnostic showed one source reporting these results under non-standard LOINCs. LA193 (1756-6, ALBUMIN) added after the A3 re-run showed it carrying serum albumin (g/dL) on its own days.</t>
         </is>
       </c>
     </row>
@@ -10566,7 +10567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M193"/>
+  <dimension ref="A1:M194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -21855,8 +21856,67 @@
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" s="5" t="inlineStr">
+        <is>
+          <t>LA193</t>
+        </is>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>ALBUMIN</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="D194" s="5" t="inlineStr">
+        <is>
+          <t>1756-6</t>
+        </is>
+      </c>
+      <c r="E194" s="5" t="inlineStr">
+        <is>
+          <t>1756-6</t>
+        </is>
+      </c>
+      <c r="F194" s="5" t="inlineStr">
+        <is>
+          <t>LAB_RESULT_CM</t>
+        </is>
+      </c>
+      <c r="G194" s="5" t="n"/>
+      <c r="H194" s="5" t="inlineStr">
+        <is>
+          <t>Albumin in CSF/Albumin in Serum or Plasma</t>
+        </is>
+      </c>
+      <c r="I194" s="5" t="inlineStr">
+        <is>
+          <t>Albumin.CSF/Albumin.SerPl</t>
+        </is>
+      </c>
+      <c r="J194" s="5" t="inlineStr">
+        <is>
+          <t>Ser/Plas+CSF</t>
+        </is>
+      </c>
+      <c r="K194" s="5" t="n"/>
+      <c r="L194" s="5" t="inlineStr">
+        <is>
+          <t>Ratio LOINC carrying a serum albumin value (unit g/dL) from one source; on 61% of sampled CMP days still missing albumin after LA191, almost never on complete days; confirmed from A3 re-run 2026-09-25</t>
+        </is>
+      </c>
+      <c r="M194" s="5" t="inlineStr">
+        <is>
+          <t>added Phase 160 from A3 missing-analyte diagnostic (second pass)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M193"/>
+  <autoFilter ref="A1:M194"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>